<commit_message>
Add Test Plan and Login Test Scenario
</commit_message>
<xml_diff>
--- a/02_Test_Plan/TestPlan.xlsx
+++ b/02_Test_Plan/TestPlan.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Manual-Tester-Portfolio\02_Test_Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FBDFA46-6E36-4CD5-AB75-EF04E173C97E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E9E6DF-A1EC-4DED-A34C-5655039557AE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4116" yWindow="1248" windowWidth="17280" windowHeight="8964" xr2:uid="{9DDF32C9-0075-4D98-AA58-ED22DD5441E8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9DDF32C9-0075-4D98-AA58-ED22DD5441E8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="TestPlan" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,9 +33,134 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+  <si>
+    <t>BOOKSTORE TEST PLAN</t>
+  </si>
+  <si>
+    <t>Project Name</t>
+  </si>
+  <si>
+    <t>BookStore</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Tester</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Build 1.0</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>Windows 11, Chrome, Excel, Postman</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>MySQL</t>
+  </si>
+  <si>
+    <t>API Tool</t>
+  </si>
+  <si>
+    <t>Postman</t>
+  </si>
+  <si>
+    <t>Test Type</t>
+  </si>
+  <si>
+    <t>Manual Testing</t>
+  </si>
+  <si>
+    <t>Test Scope</t>
+  </si>
+  <si>
+    <t>Login Module</t>
+  </si>
+  <si>
+    <t>Out of Scope</t>
+  </si>
+  <si>
+    <t>YenNhi</t>
+  </si>
+  <si>
+    <t>Test Objective</t>
+  </si>
+  <si>
+    <t>Verify Login Module satisfies all Business Rules before release.</t>
+  </si>
+  <si>
+    <t>All modules except Login.</t>
+  </si>
+  <si>
+    <t>Deliverables</t>
+  </si>
+  <si>
+    <t>Requirement Document</t>
+  </si>
+  <si>
+    <t>Requirement.xlsx</t>
+  </si>
+  <si>
+    <t>Test Scenario</t>
+  </si>
+  <si>
+    <t>TestScenario_Login.xlsx</t>
+  </si>
+  <si>
+    <t>Test Case</t>
+  </si>
+  <si>
+    <t>TestCase_Login.xlsx</t>
+  </si>
+  <si>
+    <t>Test Data</t>
+  </si>
+  <si>
+    <t>TestData_Login.xlsx</t>
+  </si>
+  <si>
+    <t>Bug Report</t>
+  </si>
+  <si>
+    <t>BugReport_Login.xlsx</t>
+  </si>
+  <si>
+    <t>SQL Verification</t>
+  </si>
+  <si>
+    <t>SQL_Verification.sql</t>
+  </si>
+  <si>
+    <t>API Testing</t>
+  </si>
+  <si>
+    <t>BookStore.postman_collection.json</t>
+  </si>
+  <si>
+    <t>Test Execution Report</t>
+  </si>
+  <si>
+    <t>Build_1.0.xlsx, Build_1.1.xlsx</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -43,16 +168,50 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -60,12 +219,106 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -380,9 +633,376 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3F30E8E-E880-4E24-BBF7-006FD62B6C31}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="12"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="12"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="12"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="12"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="12"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="12"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="12"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="40">
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="E25:H25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="E26:H26"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="E21:H21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="E22:H22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="E23:H23"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="E19:H19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="E20:H20"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E2:H2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>